<commit_message>
results colombia and cabo verde
</commit_message>
<xml_diff>
--- a/data/DRM Rapid Screening Tool - Questionnaire Cabo Verde.xlsx
+++ b/data/DRM Rapid Screening Tool - Questionnaire Cabo Verde.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="132">
   <si>
     <t xml:space="preserve">Evaluating Disaster Risk Management Policy Frameworks: A Rapid Screening Tool</t>
   </si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t xml:space="preserve">Is there a unified social registry incorporating exposure and vulnerability data to facilitate the targeting of population potentially affected in case of disaster or climate-related shocks?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partially</t>
   </si>
   <si>
     <t xml:space="preserve">Check with SP colleagues or Ministério da Família, Inclusão e Desenvolvimento Social, MFIDS</t>
@@ -1251,7 +1254,7 @@
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="18" t="str">
         <f aca="false">IF(COUNTBLANK(E15:E60)&gt;0,_xlfn.CONCAT("Please complete the assessment to proceed. Remaining questions: ",COUNTBLANK(E15:E60)), _xlfn.TEXTJOIN("&amp;",FALSE(),K15:K60))</f>
-        <v>Q1;Yes;1&amp;Q2;Yes;1&amp;Q3;Yes;1&amp;Q4;Unknown;1&amp;Q5;Yes;1&amp;Q6;Unknown;1&amp;Q7;Yes;1&amp;Q8;Unknown;1&amp;Q9;Unknown;1&amp;Q10;Unknown;1&amp;Q11;Yes;1&amp;Q12;Unknown;1&amp;Q13;Yes;1&amp;Q14;Unknown;1&amp;Q15;Yes;1&amp;Q16;Yes;1&amp;Q17;No;1&amp;Q18;Yes;0.25&amp;Q19;Unknown;0.25&amp;Q20;Unknown;0.25&amp;Q21;Unknown;0.25&amp;Q22;Yes;1&amp;Q23;Unknown;1&amp;Q24;Yes;1&amp;Q25;Yes;1&amp;Q26;Unknown;1&amp;Q27;No;1&amp;Q28;Yes;1&amp;Q29;Unknown;1&amp;Q30;Yes;1&amp;Q31;Unknown;1&amp;Q32;No;1&amp;Q33;Unknown;1&amp;Q34;Yes;1&amp;Q35;Unknown;1&amp;Q36;Unknown;1&amp;Q37;Yes;1&amp;Q38;Yes;1&amp;Q39;Yes;1&amp;Q40;Yes;1&amp;Q41;Yes;1&amp;Q42;Unknown;1&amp;Q43;Yes;1&amp;Q44;No;1&amp;Q45;No;1&amp;Q46;Yes;1</v>
+        <v>Q1;Yes;1&amp;Q2;Yes;1&amp;Q3;Yes;1&amp;Q4;Unknown;1&amp;Q5;Yes;1&amp;Q6;Unknown;1&amp;Q7;Yes;1&amp;Q8;Unknown;1&amp;Q9;Unknown;1&amp;Q10;Unknown;1&amp;Q11;Yes;1&amp;Q12;Unknown;1&amp;Q13;Yes;1&amp;Q14;Unknown;1&amp;Q15;Yes;1&amp;Q16;Yes;1&amp;Q17;No;1&amp;Q18;Yes;0.25&amp;Q19;Unknown;0.25&amp;Q20;Unknown;0.25&amp;Q21;Unknown;0.25&amp;Q22;Yes;1&amp;Q23;Unknown;1&amp;Q24;Yes;1&amp;Q25;Yes;1&amp;Q26;Unknown;1&amp;Q27;No;1&amp;Q28;Yes;1&amp;Q29;Unknown;1&amp;Q30;Yes;1&amp;Q31;Unknown;1&amp;Q32;No;1&amp;Q33;Unknown;1&amp;Q34;Yes;1&amp;Q35;Partially;1&amp;Q36;Unknown;1&amp;Q37;Yes;1&amp;Q38;Yes;1&amp;Q39;Yes;1&amp;Q40;Yes;1&amp;Q41;Yes;1&amp;Q42;Unknown;1&amp;Q43;Yes;1&amp;Q44;No;1&amp;Q45;No;1&amp;Q46;Yes;1</v>
       </c>
       <c r="C10" s="19"/>
       <c r="D10" s="20"/>
@@ -2378,11 +2381,11 @@
         <v>103</v>
       </c>
       <c r="E49" s="26" t="s">
-        <v>29</v>
+        <v>104</v>
       </c>
       <c r="F49" s="28"/>
       <c r="G49" s="28" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H49" s="29" t="n">
         <v>1</v>
@@ -2397,21 +2400,21 @@
       </c>
       <c r="K49" s="29" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J49,E49,H49)</f>
-        <v>Q35;Unknown;1</v>
+        <v>Q35;Partially;1</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="43"/>
       <c r="C50" s="24"/>
       <c r="D50" s="45" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E50" s="31" t="s">
         <v>29</v>
       </c>
       <c r="F50" s="33"/>
       <c r="G50" s="33" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H50" s="35" t="n">
         <v>1</v>
@@ -2431,19 +2434,19 @@
     </row>
     <row r="51" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="43" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C51" s="24" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D51" s="44" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E51" s="26" t="s">
         <v>21</v>
       </c>
       <c r="F51" s="28" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G51" s="28"/>
       <c r="H51" s="29" t="n">
@@ -2466,13 +2469,13 @@
       <c r="B52" s="43"/>
       <c r="C52" s="24"/>
       <c r="D52" s="45" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E52" s="31" t="s">
         <v>21</v>
       </c>
       <c r="F52" s="33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G52" s="33"/>
       <c r="H52" s="35" t="n">
@@ -2495,13 +2498,13 @@
       <c r="B53" s="43"/>
       <c r="C53" s="24"/>
       <c r="D53" s="44" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E53" s="26" t="s">
         <v>21</v>
       </c>
       <c r="F53" s="28" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G53" s="28"/>
       <c r="H53" s="29" t="n">
@@ -2524,13 +2527,13 @@
       <c r="B54" s="43"/>
       <c r="C54" s="24"/>
       <c r="D54" s="45" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E54" s="31" t="s">
         <v>21</v>
       </c>
       <c r="F54" s="33" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G54" s="33"/>
       <c r="H54" s="35" t="n">
@@ -2552,16 +2555,16 @@
     <row r="55" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="43"/>
       <c r="C55" s="24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D55" s="44" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E55" s="26" t="s">
         <v>21</v>
       </c>
       <c r="F55" s="28" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G55" s="28"/>
       <c r="H55" s="29" t="n">
@@ -2584,16 +2587,16 @@
       <c r="B56" s="43"/>
       <c r="C56" s="24"/>
       <c r="D56" s="45" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E56" s="31" t="s">
         <v>29</v>
       </c>
       <c r="F56" s="33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G56" s="33" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H56" s="35" t="n">
         <v>1</v>
@@ -2615,13 +2618,13 @@
       <c r="B57" s="43"/>
       <c r="C57" s="24"/>
       <c r="D57" s="44" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E57" s="26" t="s">
         <v>21</v>
       </c>
       <c r="F57" s="28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G57" s="28"/>
       <c r="H57" s="29" t="n">
@@ -2642,19 +2645,19 @@
     </row>
     <row r="58" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="43" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C58" s="43" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D58" s="45" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E58" s="31" t="s">
         <v>60</v>
       </c>
       <c r="F58" s="32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G58" s="33"/>
       <c r="H58" s="35" t="n">
@@ -2677,13 +2680,13 @@
       <c r="B59" s="43"/>
       <c r="C59" s="43"/>
       <c r="D59" s="44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E59" s="26" t="s">
         <v>60</v>
       </c>
       <c r="F59" s="28" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G59" s="28"/>
       <c r="H59" s="29" t="n">
@@ -2706,13 +2709,13 @@
       <c r="B60" s="43"/>
       <c r="C60" s="43"/>
       <c r="D60" s="45" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E60" s="31" t="s">
         <v>21</v>
       </c>
       <c r="F60" s="33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G60" s="46"/>
       <c r="H60" s="35" t="n">

</xml_diff>